<commit_message>
Add reviewed Scottsdale aerial replacement candidate
</commit_message>
<xml_diff>
--- a/data/airport_photo_sourcing_102_pilot.xlsx
+++ b/data/airport_photo_sourcing_102_pilot.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
@@ -582,7 +582,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>KTEB / KVNY / LFPB は各2画像、KSDLは1画像候補。KAPAの2画像とKSDLの1画像は不採用。</t>
+          <t>KTEB / KVNY / KSDL / LFPB は各2画像候補。KSDL画像1は代替空撮・承認待ち。KAPAは代替2枚未収集。</t>
         </is>
       </c>
     </row>
@@ -661,12 +661,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:H1"/>
@@ -791,7 +785,11 @@
           <t>KSDL</t>
         </is>
       </c>
-      <c r="B6" s="11" t="n"/>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/4/44/SDL_SCOTTSDALE_AIRPORT_FROM_FLIGHT_TUS-LAS_737_N748SW_%2810500329945%29_%282%29.jpg</t>
+        </is>
+      </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
           <t>https://upload.wikimedia.org/wikipedia/commons/1/11/The_Volanti_Restaurant_at_the_Scottsdale_Airport_over_looks_the_airport%E2%80%99s_runway_and_taxi_way._Camelback_Mountain_is_in_the_back_ground.jpg</t>
@@ -799,7 +797,7 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>画像1はユーザー指定で不採用。代替候補未確認。画像2は候補のまま。</t>
+          <t>画像1は代替空撮候補（2013年）。USGS航空写真と配置照合済。CC BY-SA 2.0、Eric Salardの表示等が必要。最終承認待ち。</t>
         </is>
       </c>
     </row>
@@ -2487,7 +2485,7 @@
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>1画像候補あり・1画像不採用</t>
+          <t>2画像候補あり</t>
         </is>
       </c>
       <c r="J6" s="11" t="inlineStr">
@@ -6976,7 +6974,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -7595,6 +7593,68 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>KSDL</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/4/44/SDL_SCOTTSDALE_AIRPORT_FROM_FLIGHT_TUS-LAS_737_N748SW_%2810500329945%29_%282%29.jpg</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/wiki/File:SDL_SCOTTSDALE_AIRPORT_FROM_FLIGHT_TUS-LAS_737_N748SW_(10500329945)_(2).jpg</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>SDL SCOTTSDALE AIRPORT FROM FLIGHT TUS-LAS 737 N748SW (10500329945) (2).jpg</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2308</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>1539</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>1.500</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>CC BY-SA 2.0</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Eric Salard</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2013-07-30 aerial; visually compared with independent USGS 2006 orthophoto: runway, parallel taxiways, apron and hangar blocks match. Page location differs from EXIF camera coordinates; neither alone proves location. Historical photo; credit/license link/change notice required.</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>代替候補・原画像/出典/寸法/USGS航空写真の配置照合済。用途別権利最終確認・ユーザー承認待ち</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Record two KAPA exterior candidates pending usage permission
</commit_message>
<xml_diff>
--- a/data/airport_photo_sourcing_102_pilot.xlsx
+++ b/data/airport_photo_sourcing_102_pilot.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
@@ -468,7 +468,6 @@
       <c r="G1" s="1" t="n"/>
       <c r="H1" s="1" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="21" t="inlineStr">
         <is>
@@ -513,7 +512,6 @@
         <v/>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="28" t="inlineStr">
         <is>
@@ -610,7 +608,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="19" t="inlineStr">
         <is>
@@ -659,6 +656,16 @@
         <is>
           <t>https://commons.wikimedia.org/</t>
         </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>KAPA権利確認待ち代替候補数</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -775,7 +782,7 @@
       <c r="C5" s="11" t="n"/>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>2画像ともユーザー指定で不採用。代替候補未確認。</t>
+          <t>旧2画像は不採用。代替2候補は権利/原本品質確認待ち。提出URLは未確定。</t>
         </is>
       </c>
     </row>
@@ -2435,7 +2442,7 @@
       </c>
       <c r="I5" s="11" t="inlineStr">
         <is>
-          <t>2画像とも不採用・代替未収集</t>
+          <t>代替2候補・権利/原本品質確認待ち（提出対象外）</t>
         </is>
       </c>
       <c r="J5" s="11" t="inlineStr">
@@ -6974,7 +6981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -7655,6 +7662,130 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>KAPA</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://streamline.imgix.net/8cef5e52-3c6c-4998-bf25-78e03db4b2a4/c69a48fb-f701-40ae-8227-620e2e0afa18/rs%3Dw_1200%2Ch_600%2Ccg_true%20%2811%29.webp?ixlib=rb-1.1.0&amp;w=2000&amp;h=2000&amp;fit=max&amp;or=0&amp;s=787facf38cb6e774a555e86660f4693c</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://www.centennialairport.com/discover-centennial-airport-kapa</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>rs%3Dw_1200%2Ch_600%2Ccg_true%20%2811%29.webp</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>600</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>未確認（公式サイトにCopyright表記。転載許諾なし）</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>撮影者不明。掲載者：Centennial Airport / Arapahoe County Public Airport Authority</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Runway 17L threshold and parallel taxiway, east-side apron and hangar blocks visible. Compared visually with FAA AL-5715 airport diagram and airport-published aerial PDF. Consistent layout; exact camera position not established. No camera GPS/date/author or reuse license found. Available rendition 1200x600; higher-resolution original not established.</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>代替候補・目視/寸法確認済。別資料と配置整合。権利・原本品質確認待ち、提出対象外</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>KAPA</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://streamline.imgix.net/8cef5e52-3c6c-4998-bf25-78e03db4b2a4/a96d4499-6785-4d6b-b285-954982a8406e/rs%3Dw_1200%2Ch_600%2Ccg_true%20%288%29.webp?ixlib=rb-1.1.0&amp;w=2000&amp;h=2000&amp;fit=max&amp;or=0&amp;s=a0548bc8fcf5cc13da15b0bbdc80c0f3</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://www.centennialairport.com/airport-projects</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>rs%3Dw_1200%2Ch_600%2Ccg_true%20%288%29.webp</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>600</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>未確認（公式サイトにCopyright表記。転載許諾なし）</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>撮影者不明。掲載者：Centennial Airport / Arapahoe County Public Airport Authority</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Control tower exterior with scaffolding; curved base/access road, nearby hangars and airfield visible. Tower east of main runway and north of cross runway is consistent with FAA AL-5715 and airport aerial PDF. Exact camera position/date not established. No author/reuse license found. Available rendition 1200x600; request higher-resolution original.</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>代替候補・目視/寸法確認済。別資料と配置整合。権利・原本品質確認待ち、提出対象外</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Verify KAPA candidate dimensions and public licensing evidence
</commit_message>
<xml_diff>
--- a/data/airport_photo_sourcing_102_pilot.xlsx
+++ b/data/airport_photo_sourcing_102_pilot.xlsx
@@ -7705,12 +7705,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>未確認（公式サイトにCopyright表記。転載許諾なし）</t>
+          <t>商用転載許諾を公開情報で確認できず。要権利者確認（拒否・禁止の確認ではない）</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>撮影者不明。掲載者：Centennial Airport / Arapahoe County Public Airport Authority</t>
+          <t>撮影者未確認。出典の画像キャプション空欄、配信ファイルにEXIF/XMPなし。掲載者：Centennial Airport</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -7720,7 +7720,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>代替候補・目視/寸法確認済。別資料と配置整合。権利・原本品質確認待ち、提出対象外</t>
+          <t>実寸1200×600を再検証済。商用利用許諾・高解像度原本は未確認。権利者未照会、提出対象外</t>
         </is>
       </c>
     </row>
@@ -7767,12 +7767,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>未確認（公式サイトにCopyright表記。転載許諾なし）</t>
+          <t>商用転載許諾を公開情報で確認できず。要権利者確認（拒否・禁止の確認ではない）</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>撮影者不明。掲載者：Centennial Airport / Arapahoe County Public Airport Authority</t>
+          <t>撮影者未確認。出典の画像キャプション空欄、配信ファイルにEXIF/XMPなし。掲載者：Centennial Airport</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -7782,7 +7782,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>代替候補・目視/寸法確認済。別資料と配置整合。権利・原本品質確認待ち、提出対象外</t>
+          <t>実寸1200×600を再検証済。商用利用許諾・高解像度原本は未確認。権利者未照会、提出対象外</t>
         </is>
       </c>
     </row>

</xml_diff>